<commit_message>
test: complete task-06 integration amendment and parent-resolution coverage
</commit_message>
<xml_diff>
--- a/nextseek_api/batch_upload/tests/fixtures/wave3_default_mode.xlsx
+++ b/nextseek_api/batch_upload/tests/fixtures/wave3_default_mode.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -711,18 +711,43 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>{"UID":null,"Name":"child-of-oversized","Parent":"GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_1_S13_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_2_S14_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_3_S15_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_4_S16_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_5_S17_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_6_S18_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_7_S19_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_8_S20_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_9_S21_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_10_S22_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_11_S23_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_12_S24_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_13_S25_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_14_S26_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_15_S27_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_16_S28_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_17_S29_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_18_S30_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_19_S31_L001_I1_001.fastq.gz; GBM1-DFCI4-S1to6-CSFCells-1_VDJ_IGO_16516_B_20_S32_L001_I1_001.fastq.gz"}</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>701</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Wave 3 Integration Study</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>WTNAM_blood</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>{"UID":null,"Name":"future-parent"}</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>401</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>701</v>
-      </c>
-      <c r="F12" t="inlineStr">
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>701</v>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t>Wave 3 Integration Study</t>
         </is>

</xml_diff>